<commit_message>
update data & programming.
</commit_message>
<xml_diff>
--- a/Documents/Problem 2 & 3 - Lamps.xlsx
+++ b/Documents/Problem 2 & 3 - Lamps.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/easonshao/Documents/开发/For-November-IMMC-Competition/IMMC_2022_Greater_China/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6684C34-9A0A-804E-8D02-F794259046D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B4DF5D0-2430-BF4B-A4A6-239E872D6970}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16840" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2940" yWindow="22100" windowWidth="28800" windowHeight="16840" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Basic Data" sheetId="1" r:id="rId1"/>

</xml_diff>